<commit_message>
London-Abrechnungen: CGT-Anschrift und Reisezweck ergaenzt
CGT UG, Biebricher Allee 36, 65187 Wiesbaden in beide Abrechnungen
eingetragen und im Steckbrief nachgetragen, wo Rechtsform und Sitz offen
waren. Reisezweck Messebesuch London ergaenzt; der Name der Messe fehlt
noch und steht als offener Punkt in beiden Dateien.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2Vxc1sWTkdQ9c9u5jSatw
</commit_message>
<xml_diff>
--- a/10_Output/2026-10-21-reisekosten-london-sascha-an-cgt.xlsx
+++ b/10_Output/2026-10-21-reisekosten-london-sascha-an-cgt.xlsx
@@ -169,7 +169,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="131">
   <si>
     <t xml:space="preserve">Reisekostenabrechnung</t>
   </si>
@@ -180,7 +180,7 @@
     <t xml:space="preserve">Abrechnung an</t>
   </si>
   <si>
-    <t xml:space="preserve">CGT UG</t>
+    <t xml:space="preserve">CGT UG, Biebricher Allee 36, 65187 Wiesbaden</t>
   </si>
   <si>
     <t xml:space="preserve">Gelb = ausfüllen</t>
@@ -207,6 +207,9 @@
     <t xml:space="preserve">Reisezweck</t>
   </si>
   <si>
+    <t xml:space="preserve">Messebesuch London</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kontoauszug belegt.</t>
   </si>
   <si>
@@ -420,7 +423,10 @@
     <t xml:space="preserve">OFFEN</t>
   </si>
   <si>
-    <t xml:space="preserve">Fehlt im Kopf. Ohne betrieblichen Anlass ist die Reise nicht absetzbar — Zweck und, wenn möglich, Gesprächspartner eintragen.</t>
+    <t xml:space="preserve">Welche Messe?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Im Kopf steht „Messebesuch London“. Den Namen der Messe ergänzen und die Eintrittskarte oder Registrierungsbestätigung beilegen — das ist der Nachweis des betrieblichen Anlasses, nach dem eine Prüfung als Erstes fragt.</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
@@ -1264,22 +1270,24 @@
       <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="4"/>
+      <c r="B7" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="G7" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
@@ -1287,10 +1295,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -1298,10 +1306,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
@@ -1309,10 +1317,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
@@ -1320,7 +1328,7 @@
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -1333,24 +1341,24 @@
     </row>
     <row r="14" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
@@ -1364,7 +1372,7 @@
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1377,33 +1385,33 @@
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D21" s="13" t="n">
         <v>70</v>
@@ -1474,7 +1482,7 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="16"/>
       <c r="B25" s="17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
@@ -1489,7 +1497,7 @@
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1502,27 +1510,27 @@
     </row>
     <row r="28" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B28" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D29" s="19"/>
       <c r="E29" s="19"/>
@@ -1535,13 +1543,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D30" s="19"/>
       <c r="E30" s="19"/>
@@ -1554,13 +1562,13 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D31" s="19"/>
       <c r="E31" s="19"/>
@@ -1573,13 +1581,13 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D32" s="19"/>
       <c r="E32" s="19"/>
@@ -1592,13 +1600,13 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D33" s="19"/>
       <c r="E33" s="19"/>
@@ -1611,13 +1619,13 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D34" s="19"/>
       <c r="E34" s="19"/>
@@ -1653,7 +1661,7 @@
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="16"/>
       <c r="B37" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
@@ -1668,7 +1676,7 @@
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -1681,42 +1689,42 @@
     </row>
     <row r="40" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H40" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D41" s="15" t="n">
         <f aca="false">IF($A41="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B41,'Saetze 2026'!$B$5:$B$7,0),MATCH($C41,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
@@ -1736,13 +1744,13 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D42" s="15" t="n">
         <f aca="false">IF($A42="","",IFERROR(INDEX('Saetze 2026'!$C$5:$F$7,MATCH($B42,'Saetze 2026'!$B$5:$B$7,0),MATCH($C42,'Saetze 2026'!$C$4:$F$4,0)),0))</f>
@@ -1843,7 +1851,7 @@
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="16"/>
       <c r="B47" s="17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="16"/>
@@ -1858,7 +1866,7 @@
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -1871,27 +1879,27 @@
     </row>
     <row r="50" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I50" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D51" s="19"/>
       <c r="E51" s="19"/>
@@ -1925,7 +1933,7 @@
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="16"/>
       <c r="B54" s="17" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C54" s="16"/>
       <c r="D54" s="16"/>
@@ -1940,7 +1948,7 @@
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -1953,27 +1961,27 @@
     </row>
     <row r="57" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I57" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D58" s="19"/>
       <c r="E58" s="19"/>
@@ -2020,7 +2028,7 @@
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="16"/>
       <c r="B62" s="17" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C62" s="16"/>
       <c r="D62" s="16"/>
@@ -2035,7 +2043,7 @@
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -2048,7 +2056,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B65" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="I65" s="24" t="n">
         <f aca="false">I25+I37+I47+I54+I62</f>
@@ -2057,20 +2065,20 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B66" s="25" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="I66" s="20"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B67" s="25" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I67" s="20"/>
     </row>
     <row r="68" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="26"/>
       <c r="B68" s="27" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C68" s="26"/>
       <c r="D68" s="26"/>
@@ -2085,23 +2093,23 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E71" s="25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B75" s="6"/>
       <c r="C75" s="6"/>
@@ -2114,13 +2122,13 @@
     </row>
     <row r="76" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="29" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B76" s="30" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="C76" s="31" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D76" s="31"/>
       <c r="E76" s="31"/>
@@ -2131,13 +2139,13 @@
     </row>
     <row r="77" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B77" s="33" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C77" s="34" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D77" s="34"/>
       <c r="E77" s="34"/>
@@ -2148,13 +2156,13 @@
     </row>
     <row r="78" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="29" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B78" s="30" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C78" s="31" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D78" s="31"/>
       <c r="E78" s="31"/>
@@ -2165,13 +2173,13 @@
     </row>
     <row r="79" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="29" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B79" s="30" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C79" s="31" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D79" s="31"/>
       <c r="E79" s="31"/>
@@ -2182,13 +2190,13 @@
     </row>
     <row r="80" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="29" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B80" s="30" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C80" s="31" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D80" s="31"/>
       <c r="E80" s="31"/>
@@ -2199,13 +2207,13 @@
     </row>
     <row r="81" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="29" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B81" s="30" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C81" s="31" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D81" s="31"/>
       <c r="E81" s="31"/>
@@ -2216,13 +2224,13 @@
     </row>
     <row r="82" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B82" s="33" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C82" s="34" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D82" s="34"/>
       <c r="E82" s="34"/>
@@ -2233,13 +2241,13 @@
     </row>
     <row r="83" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B83" s="33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C83" s="34" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D83" s="34"/>
       <c r="E83" s="34"/>
@@ -2250,13 +2258,13 @@
     </row>
     <row r="84" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B84" s="33" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C84" s="34" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D84" s="34"/>
       <c r="E84" s="34"/>
@@ -2267,13 +2275,13 @@
     </row>
     <row r="85" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="32" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B85" s="33" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C85" s="34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D85" s="34"/>
       <c r="E85" s="34"/>
@@ -2381,43 +2389,43 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="35" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="25" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C5" s="36" t="n">
         <v>28</v>
@@ -2432,15 +2440,15 @@
         <v>0</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C6" s="36" t="n">
         <v>66</v>
@@ -2460,10 +2468,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C7" s="36" t="n">
         <v>52</v>
@@ -2483,12 +2491,12 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B10" s="37" t="n">
         <v>0.2</v>
@@ -2496,7 +2504,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="25" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B11" s="37" t="n">
         <v>0.4</v>
@@ -2504,7 +2512,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="25" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B12" s="37" t="n">
         <v>0.4</v>
@@ -2512,12 +2520,12 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="25" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" s="38" t="n">
         <v>0.3</v>
@@ -2525,7 +2533,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="25" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C16" s="38" t="n">
         <v>0.2</v>
@@ -2533,7 +2541,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="25" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C17" s="38" t="n">
         <v>0.05</v>
@@ -2541,42 +2549,42 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>